<commit_message>
First draft of calculateResults script.
</commit_message>
<xml_diff>
--- a/analysis/resources/watchdb.all_tables.xlsx
+++ b/analysis/resources/watchdb.all_tables.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10116"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tpd0001/github/watch-wv/analysis/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF122014-041E-8E46-B55F-455066171409}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60086992-798C-814B-A30E-168E5BC209F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="960" yWindow="760" windowWidth="22700" windowHeight="18100" xr2:uid="{ABEE2980-A2EF-284E-9534-8BF6C1D1D8CC}"/>
+    <workbookView xWindow="960" yWindow="760" windowWidth="22700" windowHeight="18100" activeTab="1" xr2:uid="{ABEE2980-A2EF-284E-9534-8BF6C1D1D8CC}"/>
   </bookViews>
   <sheets>
-    <sheet name="locations" sheetId="1" r:id="rId1"/>
-    <sheet name="wwtps" sheetId="3" r:id="rId2"/>
-    <sheet name="counties" sheetId="2" r:id="rId3"/>
+    <sheet name="location" sheetId="1" r:id="rId1"/>
+    <sheet name="wwtp" sheetId="3" r:id="rId2"/>
+    <sheet name="county" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -737,9 +737,6 @@
     <t>county_name</t>
   </si>
   <si>
-    <t>primary_wwtp_id</t>
-  </si>
-  <si>
     <t>location_status</t>
   </si>
   <si>
@@ -758,9 +755,6 @@
     <t>location_comment</t>
   </si>
   <si>
-    <t>primary_lab</t>
-  </si>
-  <si>
     <t>WVU</t>
   </si>
   <si>
@@ -1128,6 +1122,12 @@
   </si>
   <si>
     <t>flow</t>
+  </si>
+  <si>
+    <t>location_primary_lab</t>
+  </si>
+  <si>
+    <t>location_primary_wwtp_id</t>
   </si>
 </sst>
 </file>
@@ -1357,7 +1357,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2013 - 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1645,7 +1645,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1677,55 +1677,55 @@
         <v>201</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>240</v>
+        <v>362</v>
       </c>
       <c r="C1" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D1" s="18" t="s">
         <v>86</v>
       </c>
       <c r="E1" s="18" t="s">
+        <v>234</v>
+      </c>
+      <c r="F1" s="18" t="s">
         <v>235</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="G1" s="20" t="s">
         <v>236</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="H1" s="18" t="s">
+        <v>363</v>
+      </c>
+      <c r="I1" s="18" t="s">
+        <v>254</v>
+      </c>
+      <c r="J1" s="21" t="s">
+        <v>253</v>
+      </c>
+      <c r="K1" s="21" t="s">
+        <v>328</v>
+      </c>
+      <c r="L1" s="21" t="s">
+        <v>356</v>
+      </c>
+      <c r="M1" s="21" t="s">
+        <v>357</v>
+      </c>
+      <c r="N1" s="21" t="s">
+        <v>358</v>
+      </c>
+      <c r="O1" s="18" t="s">
+        <v>359</v>
+      </c>
+      <c r="P1" s="18" t="s">
         <v>237</v>
-      </c>
-      <c r="H1" s="18" t="s">
-        <v>233</v>
-      </c>
-      <c r="I1" s="18" t="s">
-        <v>256</v>
-      </c>
-      <c r="J1" s="21" t="s">
-        <v>255</v>
-      </c>
-      <c r="K1" s="21" t="s">
-        <v>330</v>
-      </c>
-      <c r="L1" s="21" t="s">
-        <v>358</v>
-      </c>
-      <c r="M1" s="21" t="s">
-        <v>359</v>
-      </c>
-      <c r="N1" s="21" t="s">
-        <v>360</v>
-      </c>
-      <c r="O1" s="18" t="s">
-        <v>361</v>
-      </c>
-      <c r="P1" s="18" t="s">
-        <v>238</v>
       </c>
       <c r="Q1" s="19" t="s">
         <v>61</v>
       </c>
       <c r="R1" s="18" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -1733,7 +1733,7 @@
         <v>202</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>103</v>
@@ -1751,7 +1751,7 @@
         <v>39.637875299999997</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>11</v>
@@ -1760,7 +1760,7 @@
         <v>874</v>
       </c>
       <c r="K2" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L2" s="24">
         <v>48</v>
@@ -1772,7 +1772,7 @@
         <v>30</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>20</v>
@@ -1789,7 +1789,7 @@
         <v>31</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>103</v>
@@ -1807,16 +1807,16 @@
         <v>39.672765599999998</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J3" s="24" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="K3" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L3" s="24">
         <v>48</v>
@@ -1828,7 +1828,7 @@
         <v>30</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P3" s="2" t="s">
         <v>20</v>
@@ -1845,7 +1845,7 @@
         <v>23</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>103</v>
@@ -1863,7 +1863,7 @@
         <v>39.6511596</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>11</v>
@@ -1872,7 +1872,7 @@
         <v>862</v>
       </c>
       <c r="K4" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L4" s="24">
         <v>48</v>
@@ -1884,7 +1884,7 @@
         <v>30</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P4" s="2" t="s">
         <v>20</v>
@@ -1901,7 +1901,7 @@
         <v>194</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>103</v>
@@ -1919,7 +1919,7 @@
         <v>39.639200000000002</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>11</v>
@@ -1928,7 +1928,7 @@
         <v>474</v>
       </c>
       <c r="K5" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L5" s="24">
         <v>48</v>
@@ -1940,7 +1940,7 @@
         <v>30</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P5" s="2" t="s">
         <v>20</v>
@@ -1957,7 +1957,7 @@
         <v>24</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>103</v>
@@ -1975,7 +1975,7 @@
         <v>39.649548899999999</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>11</v>
@@ -1984,7 +1984,7 @@
         <v>904</v>
       </c>
       <c r="K6" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L6" s="24">
         <v>48</v>
@@ -1996,7 +1996,7 @@
         <v>30</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P6" s="2" t="s">
         <v>20</v>
@@ -2013,7 +2013,7 @@
         <v>32</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>103</v>
@@ -2031,16 +2031,16 @@
         <v>39.640189999999997</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J7" s="24" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="K7" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L7" s="24">
         <v>48</v>
@@ -2052,7 +2052,7 @@
         <v>30</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P7" s="2" t="s">
         <v>20</v>
@@ -2066,10 +2066,10 @@
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>103</v>
@@ -2087,16 +2087,16 @@
         <v>39.633116399999999</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J8" s="24" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="K8" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L8" s="24">
         <v>48</v>
@@ -2108,7 +2108,7 @@
         <v>30</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P8" s="2" t="s">
         <v>20</v>
@@ -2125,7 +2125,7 @@
         <v>22</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>103</v>
@@ -2134,7 +2134,7 @@
         <v>138</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="F9" s="2">
         <v>-79.972157499999994</v>
@@ -2143,16 +2143,16 @@
         <v>39.650096900000001</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J9" s="24" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="K9" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L9" s="24">
         <v>48</v>
@@ -2164,7 +2164,7 @@
         <v>30</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P9" s="2" t="s">
         <v>20</v>
@@ -2181,7 +2181,7 @@
         <v>0</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>103</v>
@@ -2190,7 +2190,7 @@
         <v>68</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F10" s="2">
         <v>-81.677679999999995</v>
@@ -2199,7 +2199,7 @@
         <v>38.372869999999999</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>1</v>
@@ -2208,7 +2208,7 @@
         <v>50000</v>
       </c>
       <c r="K10" s="23" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="L10" s="23">
         <v>24</v>
@@ -2216,7 +2216,7 @@
       <c r="M10" s="23"/>
       <c r="N10" s="23"/>
       <c r="O10" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P10" s="2" t="s">
         <v>20</v>
@@ -2231,7 +2231,7 @@
         <v>6</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>103</v>
@@ -2240,7 +2240,7 @@
         <v>69</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F11" s="2">
         <v>-77.855890000000002</v>
@@ -2249,7 +2249,7 @@
         <v>39.279240000000001</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>7</v>
@@ -2258,7 +2258,7 @@
         <v>17000</v>
       </c>
       <c r="K11" s="23" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="L11" s="23">
         <v>24</v>
@@ -2266,7 +2266,7 @@
       <c r="M11" s="23"/>
       <c r="N11" s="23"/>
       <c r="O11" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P11" s="2" t="s">
         <v>20</v>
@@ -2281,7 +2281,7 @@
         <v>93</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>103</v>
@@ -2290,7 +2290,7 @@
         <v>95</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F12" s="2">
         <v>-80.338570000000004</v>
@@ -2299,7 +2299,7 @@
         <v>39.279310000000002</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>88</v>
@@ -2308,7 +2308,7 @@
         <v>26498</v>
       </c>
       <c r="K12" s="23" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="L12" s="23">
         <v>24</v>
@@ -2316,7 +2316,7 @@
       <c r="M12" s="23"/>
       <c r="N12" s="23"/>
       <c r="O12" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P12" s="2" t="s">
         <v>20</v>
@@ -2331,7 +2331,7 @@
         <v>99</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>103</v>
@@ -2340,7 +2340,7 @@
         <v>98</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F13" s="2">
         <v>-80.018370000000004</v>
@@ -2349,7 +2349,7 @@
         <v>39.338769999999997</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>100</v>
@@ -2358,7 +2358,7 @@
         <v>6071</v>
       </c>
       <c r="K13" s="23" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="L13" s="23">
         <v>24</v>
@@ -2366,7 +2366,7 @@
       <c r="M13" s="23"/>
       <c r="N13" s="23"/>
       <c r="O13" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P13" s="2" t="s">
         <v>20</v>
@@ -2381,7 +2381,7 @@
         <v>4</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>103</v>
@@ -2390,7 +2390,7 @@
         <v>73</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F14" s="2">
         <v>-80.754930000000002</v>
@@ -2399,7 +2399,7 @@
         <v>39.929859999999998</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>5</v>
@@ -2408,7 +2408,7 @@
         <v>12000</v>
       </c>
       <c r="K14" s="23" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="L14" s="23">
         <v>24</v>
@@ -2416,7 +2416,7 @@
       <c r="M14" s="23"/>
       <c r="N14" s="23"/>
       <c r="O14" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P14" s="2" t="s">
         <v>20</v>
@@ -2431,7 +2431,7 @@
         <v>49</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>103</v>
@@ -2440,7 +2440,7 @@
         <v>76</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F15" s="2">
         <v>-81.557389999999998</v>
@@ -2449,7 +2449,7 @@
         <v>39.281709999999997</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>54</v>
@@ -2458,7 +2458,7 @@
         <v>48050</v>
       </c>
       <c r="K15" s="23" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="L15" s="23">
         <v>24</v>
@@ -2466,7 +2466,7 @@
       <c r="M15" s="23"/>
       <c r="N15" s="23"/>
       <c r="O15" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P15" s="2" t="s">
         <v>20</v>
@@ -2481,7 +2481,7 @@
         <v>10</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>103</v>
@@ -2490,7 +2490,7 @@
         <v>137</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F16" s="2">
         <v>-79.992055399999998</v>
@@ -2499,7 +2499,7 @@
         <v>39.655174500000001</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>11</v>
@@ -2508,7 +2508,7 @@
         <v>48328</v>
       </c>
       <c r="K16" s="23" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="L16" s="23">
         <v>24</v>
@@ -2516,7 +2516,7 @@
       <c r="M16" s="23"/>
       <c r="N16" s="23"/>
       <c r="O16" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P16" s="2" t="s">
         <v>20</v>
@@ -2531,7 +2531,7 @@
         <v>2</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>103</v>
@@ -2540,7 +2540,7 @@
         <v>85</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F17" s="2">
         <v>-80.72757</v>
@@ -2549,7 +2549,7 @@
         <v>40.055880000000002</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>3</v>
@@ -2558,7 +2558,7 @@
         <v>50000</v>
       </c>
       <c r="K17" s="23" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="L17" s="23">
         <v>24</v>
@@ -2566,7 +2566,7 @@
       <c r="M17" s="23"/>
       <c r="N17" s="23"/>
       <c r="O17" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P17" s="2" t="s">
         <v>20</v>
@@ -2581,7 +2581,7 @@
         <v>62</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>103</v>
@@ -2590,7 +2590,7 @@
         <v>64</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F18" s="2">
         <v>-79.50179</v>
@@ -2599,7 +2599,7 @@
         <v>39.457090000000001</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>63</v>
@@ -2609,7 +2609,7 @@
         <v>700</v>
       </c>
       <c r="K18" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L18" s="23">
         <v>24</v>
@@ -2621,7 +2621,7 @@
         <v>20</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P18" s="2" t="s">
         <v>20</v>
@@ -2636,7 +2636,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>103</v>
@@ -2645,7 +2645,7 @@
         <v>65</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F19" s="2">
         <v>-81.015979999999999</v>
@@ -2654,7 +2654,7 @@
         <v>37.42163</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>17</v>
@@ -2663,7 +2663,7 @@
         <v>2391</v>
       </c>
       <c r="K19" s="24" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="L19" s="23">
         <v>24</v>
@@ -2675,7 +2675,7 @@
         <v>20</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P19" s="2" t="s">
         <v>20</v>
@@ -2690,7 +2690,7 @@
         <v>101</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>103</v>
@@ -2699,7 +2699,7 @@
         <v>102</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F20" s="2">
         <v>-79.856999999999999</v>
@@ -2708,7 +2708,7 @@
         <v>39.677120000000002</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>11</v>
@@ -2717,7 +2717,7 @@
         <v>2000</v>
       </c>
       <c r="K20" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L20" s="23">
         <v>24</v>
@@ -2729,7 +2729,7 @@
         <v>20</v>
       </c>
       <c r="O20" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P20" s="2" t="s">
         <v>20</v>
@@ -2744,7 +2744,7 @@
         <v>113</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>103</v>
@@ -2753,7 +2753,7 @@
         <v>120</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F21" s="2">
         <v>-79.865430000000003</v>
@@ -2762,7 +2762,7 @@
         <v>38.920259999999999</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>121</v>
@@ -2771,7 +2771,7 @@
         <v>13156</v>
       </c>
       <c r="K21" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L21" s="23">
         <v>24</v>
@@ -2783,7 +2783,7 @@
         <v>20</v>
       </c>
       <c r="O21" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P21" s="2" t="s">
         <v>20</v>
@@ -2797,7 +2797,7 @@
         <v>109</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>103</v>
@@ -2806,7 +2806,7 @@
         <v>116</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F22" s="2">
         <v>-80.24933</v>
@@ -2815,7 +2815,7 @@
         <v>39.511809999999997</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>89</v>
@@ -2824,7 +2824,7 @@
         <v>610</v>
       </c>
       <c r="K22" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L22" s="23">
         <v>24</v>
@@ -2836,7 +2836,7 @@
         <v>20</v>
       </c>
       <c r="O22" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P22" s="2" t="s">
         <v>20</v>
@@ -2851,7 +2851,7 @@
         <v>111</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>103</v>
@@ -2860,7 +2860,7 @@
         <v>118</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F23" s="2">
         <v>-80.598290000000006</v>
@@ -2869,7 +2869,7 @@
         <v>40.325800000000001</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>122</v>
@@ -2878,7 +2878,7 @@
         <v>6468</v>
       </c>
       <c r="K23" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L23" s="23">
         <v>24</v>
@@ -2890,7 +2890,7 @@
         <v>20</v>
       </c>
       <c r="O23" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P23" s="2" t="s">
         <v>20</v>
@@ -2904,7 +2904,7 @@
         <v>108</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>103</v>
@@ -2913,7 +2913,7 @@
         <v>115</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F24" s="2">
         <v>-79.978949999999998</v>
@@ -2922,7 +2922,7 @@
         <v>38.712879999999998</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>121</v>
@@ -2931,7 +2931,7 @@
         <v>2101</v>
       </c>
       <c r="K24" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L24" s="23">
         <v>24</v>
@@ -2943,7 +2943,7 @@
         <v>20</v>
       </c>
       <c r="O24" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P24" s="2" t="s">
         <v>20</v>
@@ -2958,7 +2958,7 @@
         <v>12</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>103</v>
@@ -2967,7 +2967,7 @@
         <v>71</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F25" s="2">
         <v>-78.975080000000005</v>
@@ -2976,7 +2976,7 @@
         <v>39.441229999999997</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>13</v>
@@ -2985,7 +2985,7 @@
         <v>8168</v>
       </c>
       <c r="K25" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L25" s="23">
         <v>24</v>
@@ -2997,7 +2997,7 @@
         <v>20</v>
       </c>
       <c r="O25" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P25" s="2" t="s">
         <v>20</v>
@@ -3011,7 +3011,7 @@
         <v>152</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>103</v>
@@ -3020,7 +3020,7 @@
         <v>154</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F26" s="2">
         <v>-81.847288800000001</v>
@@ -3029,7 +3029,7 @@
         <v>38.102483999999997</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>153</v>
@@ -3038,7 +3038,7 @@
         <v>4555</v>
       </c>
       <c r="K26" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L26" s="23">
         <v>24</v>
@@ -3050,7 +3050,7 @@
         <v>20</v>
       </c>
       <c r="O26" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P26" s="2" t="s">
         <v>20</v>
@@ -3065,7 +3065,7 @@
         <v>104</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>103</v>
@@ -3074,7 +3074,7 @@
         <v>105</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F27" s="2">
         <v>-80.323710000000005</v>
@@ -3083,7 +3083,7 @@
         <v>39.518140000000002</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>89</v>
@@ -3092,7 +3092,7 @@
         <v>1091</v>
       </c>
       <c r="K27" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L27" s="23">
         <v>24</v>
@@ -3104,7 +3104,7 @@
         <v>20</v>
       </c>
       <c r="O27" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P27" s="2" t="s">
         <v>20</v>
@@ -3119,7 +3119,7 @@
         <v>198</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>103</v>
@@ -3128,7 +3128,7 @@
         <v>199</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F28" s="2">
         <v>-82.135114799999997</v>
@@ -3137,7 +3137,7 @@
         <v>38.856708400000002</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>200</v>
@@ -3146,7 +3146,7 @@
         <v>5515</v>
       </c>
       <c r="K28" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L28" s="23">
         <v>24</v>
@@ -3158,7 +3158,7 @@
         <v>20</v>
       </c>
       <c r="O28" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P28" s="2" t="s">
         <v>20</v>
@@ -3173,7 +3173,7 @@
         <v>16</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>103</v>
@@ -3182,7 +3182,7 @@
         <v>78</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F29" s="2">
         <v>-81.079930000000004</v>
@@ -3191,7 +3191,7 @@
         <v>37.380360000000003</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>17</v>
@@ -3200,7 +3200,7 @@
         <v>36000</v>
       </c>
       <c r="K29" s="24" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="L29" s="23">
         <v>24</v>
@@ -3212,7 +3212,7 @@
         <v>20</v>
       </c>
       <c r="O29" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P29" s="2" t="s">
         <v>20</v>
@@ -3227,7 +3227,7 @@
         <v>106</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>103</v>
@@ -3236,7 +3236,7 @@
         <v>107</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F30" s="2">
         <v>-80.545150000000007</v>
@@ -3245,7 +3245,7 @@
         <v>39.285969999999999</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>88</v>
@@ -3254,7 +3254,7 @@
         <v>1853</v>
       </c>
       <c r="K30" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L30" s="23">
         <v>24</v>
@@ -3266,7 +3266,7 @@
         <v>20</v>
       </c>
       <c r="O30" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P30" s="2" t="s">
         <v>20</v>
@@ -3281,7 +3281,7 @@
         <v>51</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>103</v>
@@ -3290,7 +3290,7 @@
         <v>79</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F31" s="2">
         <v>-81.205110000000005</v>
@@ -3299,7 +3299,7 @@
         <v>39.391249999999999</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="I31" s="2" t="s">
         <v>56</v>
@@ -3308,7 +3308,7 @@
         <v>2892</v>
       </c>
       <c r="K31" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L31" s="23">
         <v>24</v>
@@ -3320,7 +3320,7 @@
         <v>20</v>
       </c>
       <c r="O31" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P31" s="2" t="s">
         <v>20</v>
@@ -3335,7 +3335,7 @@
         <v>8</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>103</v>
@@ -3344,7 +3344,7 @@
         <v>83</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F32" s="2">
         <v>-80.459909999999994</v>
@@ -3353,7 +3353,7 @@
         <v>39.062240000000003</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="I32" s="2" t="s">
         <v>9</v>
@@ -3362,7 +3362,7 @@
         <v>10364</v>
       </c>
       <c r="K32" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L32" s="23">
         <v>24</v>
@@ -3374,7 +3374,7 @@
         <v>20</v>
       </c>
       <c r="O32" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P32" s="2" t="s">
         <v>20</v>
@@ -3389,7 +3389,7 @@
         <v>52</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>103</v>
@@ -3398,7 +3398,7 @@
         <v>84</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F33" s="2">
         <v>-80.778989999999993</v>
@@ -3407,7 +3407,7 @@
         <v>39.299059999999997</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="I33" s="2" t="s">
         <v>57</v>
@@ -3416,7 +3416,7 @@
         <v>564</v>
       </c>
       <c r="K33" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L33" s="23">
         <v>24</v>
@@ -3428,7 +3428,7 @@
         <v>20</v>
       </c>
       <c r="O33" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P33" s="2" t="s">
         <v>20</v>
@@ -3440,10 +3440,10 @@
     </row>
     <row r="34" spans="1:18" s="9" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>60</v>
@@ -3461,7 +3461,7 @@
         <v>39.66807</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="I34" s="2" t="s">
         <v>63</v>
@@ -3470,15 +3470,15 @@
         <v>1948</v>
       </c>
       <c r="K34" s="23" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="L34" s="23" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="M34" s="23"/>
       <c r="N34" s="23"/>
       <c r="O34" s="2" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="P34" s="2" t="s">
         <v>20</v>
@@ -3493,7 +3493,7 @@
         <v>21</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>60</v>
@@ -3511,7 +3511,7 @@
         <v>39.6362083</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I35" s="2" t="s">
         <v>11</v>
@@ -3520,7 +3520,7 @@
         <v>567</v>
       </c>
       <c r="K35" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L35" s="24">
         <v>48</v>
@@ -3532,7 +3532,7 @@
         <v>30</v>
       </c>
       <c r="O35" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P35" s="2" t="s">
         <v>20</v>
@@ -3549,7 +3549,7 @@
         <v>25</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>60</v>
@@ -3567,7 +3567,7 @@
         <v>39.636423100000002</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I36" s="2" t="s">
         <v>11</v>
@@ -3576,7 +3576,7 @@
         <v>639</v>
       </c>
       <c r="K36" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L36" s="24">
         <v>48</v>
@@ -3588,7 +3588,7 @@
         <v>30</v>
       </c>
       <c r="O36" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P36" s="2" t="s">
         <v>20</v>
@@ -3605,7 +3605,7 @@
         <v>26</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>60</v>
@@ -3623,7 +3623,7 @@
         <v>39.6535571</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I37" s="2" t="s">
         <v>11</v>
@@ -3632,7 +3632,7 @@
         <v>912</v>
       </c>
       <c r="K37" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L37" s="24">
         <v>48</v>
@@ -3644,7 +3644,7 @@
         <v>30</v>
       </c>
       <c r="O37" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P37" s="2" t="s">
         <v>20</v>
@@ -3661,7 +3661,7 @@
         <v>27</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>60</v>
@@ -3679,16 +3679,16 @@
         <v>39.667909799999997</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I38" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J38" s="24" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="K38" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L38" s="24">
         <v>48</v>
@@ -3700,7 +3700,7 @@
         <v>30</v>
       </c>
       <c r="O38" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P38" s="2" t="s">
         <v>20</v>
@@ -3717,7 +3717,7 @@
         <v>28</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>60</v>
@@ -3735,16 +3735,16 @@
         <v>39.668112200000003</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I39" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J39" s="24" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="K39" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L39" s="24">
         <v>48</v>
@@ -3756,7 +3756,7 @@
         <v>30</v>
       </c>
       <c r="O39" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P39" s="2" t="s">
         <v>20</v>
@@ -3773,7 +3773,7 @@
         <v>29</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>60</v>
@@ -3791,16 +3791,16 @@
         <v>39.669188599999998</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J40" s="24" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="K40" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L40" s="24">
         <v>48</v>
@@ -3812,7 +3812,7 @@
         <v>30</v>
       </c>
       <c r="O40" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P40" s="2" t="s">
         <v>20</v>
@@ -3829,7 +3829,7 @@
         <v>30</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>60</v>
@@ -3847,16 +3847,16 @@
         <v>39.669279500000002</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I41" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J41" s="24" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="K41" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L41" s="24">
         <v>48</v>
@@ -3868,7 +3868,7 @@
         <v>30</v>
       </c>
       <c r="O41" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P41" s="2" t="s">
         <v>20</v>
@@ -3885,7 +3885,7 @@
         <v>33</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>60</v>
@@ -3903,16 +3903,16 @@
         <v>39.6565887</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I42" s="2" t="s">
         <v>11</v>
       </c>
       <c r="J42" s="24" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="K42" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L42" s="24">
         <v>48</v>
@@ -3924,7 +3924,7 @@
         <v>30</v>
       </c>
       <c r="O42" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P42" s="2" t="s">
         <v>20</v>
@@ -3941,7 +3941,7 @@
         <v>58</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>60</v>
@@ -3959,7 +3959,7 @@
         <v>39.671370000000003</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I43" s="2" t="s">
         <v>11</v>
@@ -3968,7 +3968,7 @@
         <v>515</v>
       </c>
       <c r="K43" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L43" s="24">
         <v>8</v>
@@ -3976,7 +3976,7 @@
       <c r="M43" s="24"/>
       <c r="N43" s="24"/>
       <c r="O43" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P43" s="2" t="s">
         <v>20</v>
@@ -3990,7 +3990,7 @@
         <v>35</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>60</v>
@@ -4008,7 +4008,7 @@
         <v>39.610210000000002</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I44" s="2" t="s">
         <v>11</v>
@@ -4017,7 +4017,7 @@
         <v>579</v>
       </c>
       <c r="K44" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L44" s="24">
         <v>8</v>
@@ -4025,7 +4025,7 @@
       <c r="M44" s="24"/>
       <c r="N44" s="24"/>
       <c r="O44" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P44" s="2" t="s">
         <v>20</v>
@@ -4039,7 +4039,7 @@
         <v>40</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>60</v>
@@ -4057,7 +4057,7 @@
         <v>39.652670000000001</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I45" s="2" t="s">
         <v>11</v>
@@ -4066,7 +4066,7 @@
         <v>830</v>
       </c>
       <c r="K45" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L45" s="24">
         <v>8</v>
@@ -4074,7 +4074,7 @@
       <c r="M45" s="24"/>
       <c r="N45" s="24"/>
       <c r="O45" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P45" s="2" t="s">
         <v>20</v>
@@ -4088,7 +4088,7 @@
         <v>38</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>60</v>
@@ -4106,7 +4106,7 @@
         <v>39.625419999999998</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I46" s="2" t="s">
         <v>11</v>
@@ -4115,7 +4115,7 @@
         <v>1851</v>
       </c>
       <c r="K46" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L46" s="24">
         <v>8</v>
@@ -4123,7 +4123,7 @@
       <c r="M46" s="24"/>
       <c r="N46" s="24"/>
       <c r="O46" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P46" s="2" t="s">
         <v>20</v>
@@ -4137,7 +4137,7 @@
         <v>39</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>60</v>
@@ -4155,7 +4155,7 @@
         <v>39.61036</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I47" s="2" t="s">
         <v>11</v>
@@ -4164,7 +4164,7 @@
         <v>726</v>
       </c>
       <c r="K47" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L47" s="24">
         <v>8</v>
@@ -4172,7 +4172,7 @@
       <c r="M47" s="24"/>
       <c r="N47" s="24"/>
       <c r="O47" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P47" s="2" t="s">
         <v>20</v>
@@ -4186,7 +4186,7 @@
         <v>36</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C48" s="4" t="s">
         <v>60</v>
@@ -4204,7 +4204,7 @@
         <v>39.660640000000001</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I48" s="2" t="s">
         <v>11</v>
@@ -4213,7 +4213,7 @@
         <v>688</v>
       </c>
       <c r="K48" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L48" s="24">
         <v>8</v>
@@ -4221,7 +4221,7 @@
       <c r="M48" s="24"/>
       <c r="N48" s="24"/>
       <c r="O48" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P48" s="2" t="s">
         <v>20</v>
@@ -4235,7 +4235,7 @@
         <v>37</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C49" s="4" t="s">
         <v>60</v>
@@ -4253,7 +4253,7 @@
         <v>39.687820000000002</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I49" s="2" t="s">
         <v>11</v>
@@ -4262,7 +4262,7 @@
         <v>1310</v>
       </c>
       <c r="K49" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L49" s="24">
         <v>8</v>
@@ -4270,7 +4270,7 @@
       <c r="M49" s="24"/>
       <c r="N49" s="24"/>
       <c r="O49" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P49" s="2" t="s">
         <v>20</v>
@@ -4284,7 +4284,7 @@
         <v>50</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>60</v>
@@ -4293,7 +4293,7 @@
         <v>77</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F50" s="2">
         <v>-79.127250000000004</v>
@@ -4302,7 +4302,7 @@
         <v>38.99091</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="I50" s="2" t="s">
         <v>55</v>
@@ -4311,7 +4311,7 @@
         <v>2700</v>
       </c>
       <c r="K50" s="23" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="L50" s="23">
         <v>24</v>
@@ -4319,7 +4319,7 @@
       <c r="M50" s="23"/>
       <c r="N50" s="23"/>
       <c r="O50" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P50" s="2" t="s">
         <v>20</v>
@@ -4333,7 +4333,7 @@
         <v>182</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>60</v>
@@ -4362,7 +4362,7 @@
         <v>188</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C52" s="4" t="s">
         <v>60</v>
@@ -4391,7 +4391,7 @@
         <v>184</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C53" s="4" t="s">
         <v>60</v>
@@ -4420,7 +4420,7 @@
         <v>186</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C54" s="4" t="s">
         <v>60</v>
@@ -4449,7 +4449,7 @@
         <v>173</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>60</v>
@@ -4458,7 +4458,7 @@
         <v>68</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F55" s="2">
         <v>-81.679554234298493</v>
@@ -4476,7 +4476,7 @@
         <v>49500</v>
       </c>
       <c r="K55" s="23" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="L55" s="23">
         <v>24</v>
@@ -4484,7 +4484,7 @@
       <c r="M55" s="23"/>
       <c r="N55" s="23"/>
       <c r="O55" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P55" s="2" t="s">
         <v>20</v>
@@ -4498,7 +4498,7 @@
         <v>181</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C56" s="4" t="s">
         <v>60</v>
@@ -4507,7 +4507,7 @@
         <v>164</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F56" s="2">
         <v>-81.758709180509001</v>
@@ -4525,7 +4525,7 @@
         <v>9000</v>
       </c>
       <c r="K56" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L56" s="23">
         <v>24</v>
@@ -4537,7 +4537,7 @@
         <v>20</v>
       </c>
       <c r="O56" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P56" s="2" t="s">
         <v>20</v>
@@ -4552,7 +4552,7 @@
         <v>175</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>60</v>
@@ -4561,7 +4561,7 @@
         <v>160</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F57" s="2">
         <v>-82.006959612418996</v>
@@ -4579,7 +4579,7 @@
         <v>28759</v>
       </c>
       <c r="K57" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L57" s="23">
         <v>24</v>
@@ -4591,7 +4591,7 @@
         <v>20</v>
       </c>
       <c r="O57" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P57" s="2" t="s">
         <v>20</v>
@@ -4606,7 +4606,7 @@
         <v>172</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C58" s="4" t="s">
         <v>60</v>
@@ -4615,7 +4615,7 @@
         <v>155</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F58" s="2">
         <v>-82.528864034905197</v>
@@ -4633,7 +4633,7 @@
         <v>56000</v>
       </c>
       <c r="K58" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L58" s="23">
         <v>24</v>
@@ -4645,7 +4645,7 @@
         <v>20</v>
       </c>
       <c r="O58" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P58" s="2" t="s">
         <v>20</v>
@@ -4660,7 +4660,7 @@
         <v>165</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>60</v>
@@ -4669,7 +4669,7 @@
         <v>166</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F59" s="2">
         <v>-82.451303840583293</v>
@@ -4687,7 +4687,7 @@
         <v>1600</v>
       </c>
       <c r="K59" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L59" s="23">
         <v>24</v>
@@ -4699,7 +4699,7 @@
         <v>20</v>
       </c>
       <c r="O59" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P59" s="2" t="s">
         <v>20</v>
@@ -4716,7 +4716,7 @@
         <v>169</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>60</v>
@@ -4725,7 +4725,7 @@
         <v>170</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F60" s="2">
         <v>-82.287563960345196</v>
@@ -4743,7 +4743,7 @@
         <v>1000</v>
       </c>
       <c r="K60" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L60" s="23">
         <v>24</v>
@@ -4755,7 +4755,7 @@
         <v>20</v>
       </c>
       <c r="O60" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P60" s="2" t="s">
         <v>20</v>
@@ -4772,7 +4772,7 @@
         <v>180</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>60</v>
@@ -4781,7 +4781,7 @@
         <v>163</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F61" s="2">
         <v>-82.298209254857795</v>
@@ -4799,7 +4799,7 @@
         <v>7000</v>
       </c>
       <c r="K61" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L61" s="23">
         <v>24</v>
@@ -4811,7 +4811,7 @@
         <v>20</v>
       </c>
       <c r="O61" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P61" s="2" t="s">
         <v>20</v>
@@ -4826,7 +4826,7 @@
         <v>178</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C62" s="4" t="s">
         <v>60</v>
@@ -4835,7 +4835,7 @@
         <v>179</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F62" s="2">
         <v>-82.209446953848399</v>
@@ -4853,7 +4853,7 @@
         <v>11250</v>
       </c>
       <c r="K62" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L62" s="23">
         <v>24</v>
@@ -4865,7 +4865,7 @@
         <v>20</v>
       </c>
       <c r="O62" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P62" s="2" t="s">
         <v>20</v>
@@ -4882,7 +4882,7 @@
         <v>176</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>60</v>
@@ -4891,7 +4891,7 @@
         <v>177</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F63" s="2">
         <v>-82.209446953848399</v>
@@ -4909,7 +4909,7 @@
         <v>11250</v>
       </c>
       <c r="K63" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L63" s="23">
         <v>24</v>
@@ -4921,7 +4921,7 @@
         <v>20</v>
       </c>
       <c r="O63" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P63" s="2" t="s">
         <v>20</v>
@@ -4938,7 +4938,7 @@
         <v>174</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C64" s="4" t="s">
         <v>60</v>
@@ -4947,7 +4947,7 @@
         <v>156</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F64" s="2">
         <v>-82.285698770801503</v>
@@ -4966,7 +4966,7 @@
       </c>
       <c r="K64" s="24"/>
       <c r="L64" s="24" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="M64" s="24"/>
       <c r="N64" s="24"/>
@@ -4988,7 +4988,7 @@
         <v>59</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C65" s="4" t="s">
         <v>190</v>
@@ -5006,7 +5006,7 @@
         <v>39.438070000000003</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="I65" s="2" t="s">
         <v>13</v>
@@ -5015,7 +5015,7 @@
         <v>1193</v>
       </c>
       <c r="K65" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L65" s="24">
         <v>48</v>
@@ -5027,7 +5027,7 @@
         <v>30</v>
       </c>
       <c r="O65" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P65" s="2" t="s">
         <v>20</v>
@@ -5042,7 +5042,7 @@
         <v>112</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C66" s="4" t="s">
         <v>190</v>
@@ -5051,7 +5051,7 @@
         <v>119</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F66" s="2">
         <v>-79.936940000000007</v>
@@ -5060,7 +5060,7 @@
         <v>39.022010000000002</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I66" s="2" t="s">
         <v>123</v>
@@ -5069,7 +5069,7 @@
         <v>1974</v>
       </c>
       <c r="K66" s="23" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="L66" s="23">
         <v>24</v>
@@ -5077,7 +5077,7 @@
       <c r="M66" s="23"/>
       <c r="N66" s="23"/>
       <c r="O66" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P66" s="2" t="s">
         <v>20</v>
@@ -5092,7 +5092,7 @@
         <v>110</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C67" s="4" t="s">
         <v>190</v>
@@ -5101,7 +5101,7 @@
         <v>117</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F67" s="2">
         <v>-80.212010000000006</v>
@@ -5110,7 +5110,7 @@
         <v>39.72007</v>
       </c>
       <c r="H67" s="2" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="I67" s="2" t="s">
         <v>11</v>
@@ -5119,7 +5119,7 @@
         <v>400</v>
       </c>
       <c r="K67" s="23" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="L67" s="23">
         <v>24</v>
@@ -5127,7 +5127,7 @@
       <c r="M67" s="23"/>
       <c r="N67" s="23"/>
       <c r="O67" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P67" s="2" t="s">
         <v>20</v>
@@ -5142,7 +5142,7 @@
         <v>92</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C68" s="4" t="s">
         <v>190</v>
@@ -5151,7 +5151,7 @@
         <v>94</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F68" s="2">
         <v>-80.258989999999997</v>
@@ -5160,7 +5160,7 @@
         <v>39.280479999999997</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="I68" s="2" t="s">
         <v>88</v>
@@ -5169,7 +5169,7 @@
         <v>6984</v>
       </c>
       <c r="K68" s="23" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="L68" s="23">
         <v>24</v>
@@ -5177,7 +5177,7 @@
       <c r="M68" s="23"/>
       <c r="N68" s="23"/>
       <c r="O68" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P68" s="2" t="s">
         <v>20</v>
@@ -5192,7 +5192,7 @@
         <v>125</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C69" s="4" t="s">
         <v>190</v>
@@ -5201,12 +5201,12 @@
         <v>128</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F69" s="2"/>
       <c r="G69" s="2"/>
       <c r="H69" s="2" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="I69" s="2" t="s">
         <v>129</v>
@@ -5215,7 +5215,7 @@
         <v>1800</v>
       </c>
       <c r="K69" s="23" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="L69" s="23">
         <v>24</v>
@@ -5223,7 +5223,7 @@
       <c r="M69" s="23"/>
       <c r="N69" s="23"/>
       <c r="O69" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P69" s="2" t="s">
         <v>20</v>
@@ -5236,7 +5236,7 @@
         <v>14</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C70" s="4" t="s">
         <v>190</v>
@@ -5245,7 +5245,7 @@
         <v>82</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F70" s="2">
         <v>-78.226619999999997</v>
@@ -5254,7 +5254,7 @@
         <v>39.628019999999999</v>
       </c>
       <c r="H70" s="2" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I70" s="2" t="s">
         <v>15</v>
@@ -5263,7 +5263,7 @@
         <v>3255</v>
       </c>
       <c r="K70" s="23" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="L70" s="23">
         <v>24</v>
@@ -5271,7 +5271,7 @@
       <c r="M70" s="23"/>
       <c r="N70" s="23"/>
       <c r="O70" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P70" s="2" t="s">
         <v>20</v>
@@ -5286,7 +5286,7 @@
         <v>126</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C71" s="4" t="s">
         <v>190</v>
@@ -5295,12 +5295,12 @@
         <v>127</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F71" s="2"/>
       <c r="G71" s="2"/>
       <c r="H71" s="2" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="I71" s="2" t="s">
         <v>122</v>
@@ -5309,7 +5309,7 @@
         <v>20411</v>
       </c>
       <c r="K71" s="23" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="L71" s="23">
         <v>24</v>
@@ -5317,7 +5317,7 @@
       <c r="M71" s="23"/>
       <c r="N71" s="23"/>
       <c r="O71" s="2" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="P71" s="2" t="s">
         <v>20</v>
@@ -5330,7 +5330,7 @@
         <v>53</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C72" s="4" t="s">
         <v>190</v>
@@ -5339,7 +5339,7 @@
         <v>67</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F72" s="2">
         <v>-80.567440000000005</v>
@@ -5348,7 +5348,7 @@
         <v>39.826610000000002</v>
       </c>
       <c r="H72" s="2" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="I72" s="2" t="s">
         <v>5</v>
@@ -5357,7 +5357,7 @@
         <v>1340</v>
       </c>
       <c r="K72" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L72" s="23">
         <v>24</v>
@@ -5369,7 +5369,7 @@
         <v>30</v>
       </c>
       <c r="O72" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P72" s="2" t="s">
         <v>20</v>
@@ -5384,7 +5384,7 @@
         <v>91</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C73" s="4" t="s">
         <v>190</v>
@@ -5393,7 +5393,7 @@
         <v>97</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F73" s="2">
         <v>-80.124449999999996</v>
@@ -5402,7 +5402,7 @@
         <v>39.493949999999998</v>
       </c>
       <c r="H73" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="I73" s="2" t="s">
         <v>89</v>
@@ -5411,7 +5411,7 @@
         <v>25525</v>
       </c>
       <c r="K73" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L73" s="23">
         <v>24</v>
@@ -5423,7 +5423,7 @@
         <v>30</v>
       </c>
       <c r="O73" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P73" s="2" t="s">
         <v>20</v>
@@ -5438,7 +5438,7 @@
         <v>90</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C74" s="4" t="s">
         <v>190</v>
@@ -5447,7 +5447,7 @@
         <v>96</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="F74" s="2">
         <v>-80.260360000000006</v>
@@ -5456,7 +5456,7 @@
         <v>39.452579999999998</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="I74" s="2" t="s">
         <v>89</v>
@@ -5465,7 +5465,7 @@
         <v>2742</v>
       </c>
       <c r="K74" s="24" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="L74" s="23">
         <v>24</v>
@@ -5477,7 +5477,7 @@
         <v>30</v>
       </c>
       <c r="O74" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P74" s="2" t="s">
         <v>20</v>
@@ -5511,36 +5511,36 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="12" t="s">
+        <v>242</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>249</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="G1" s="13" t="s">
         <v>244</v>
-      </c>
-      <c r="B1" s="12" t="s">
-        <v>243</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>251</v>
-      </c>
-      <c r="D1" s="12" t="s">
-        <v>252</v>
-      </c>
-      <c r="E1" s="12" t="s">
-        <v>254</v>
-      </c>
-      <c r="F1" s="13" t="s">
-        <v>247</v>
-      </c>
-      <c r="G1" s="13" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="14" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B2" s="14" t="s">
         <v>64</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>63</v>
@@ -5558,13 +5558,13 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>17</v>
@@ -5581,13 +5581,13 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="14" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>123</v>
@@ -5604,13 +5604,13 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>11</v>
@@ -5627,13 +5627,13 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>88</v>
@@ -5669,10 +5669,10 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="14" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C8" s="14"/>
       <c r="D8" s="14" t="s">
@@ -5688,10 +5688,10 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="14" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="14" t="s">
@@ -5707,10 +5707,10 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="14" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="14" t="s">
@@ -5726,13 +5726,13 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="14" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D11" s="14" t="s">
         <v>11</v>
@@ -5749,10 +5749,10 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="14" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C12" s="14"/>
       <c r="D12" s="14" t="s">
@@ -5806,10 +5806,10 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="14" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C15" s="14"/>
       <c r="D15" s="14" t="s">
@@ -5825,10 +5825,10 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="14" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C16" s="14"/>
       <c r="D16" s="14" t="s">
@@ -5844,10 +5844,10 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="14" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C17" s="14"/>
       <c r="D17" s="14" t="s">
@@ -5863,10 +5863,10 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="14" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C18" s="14"/>
       <c r="D18" s="14" t="s">
@@ -5882,10 +5882,10 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="14" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C19" s="14"/>
       <c r="D19" s="14" t="s">
@@ -5901,13 +5901,13 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="14" t="s">
+        <v>246</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>302</v>
+      </c>
+      <c r="C20" s="14" t="s">
         <v>248</v>
-      </c>
-      <c r="B20" s="14" t="s">
-        <v>304</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>250</v>
       </c>
       <c r="D20" s="14" t="s">
         <v>63</v>
@@ -5943,10 +5943,10 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="14" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C22" s="14"/>
       <c r="D22" s="14" t="s">
@@ -5962,10 +5962,10 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="14" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C23" s="14"/>
       <c r="D23" s="14" t="s">
@@ -5981,10 +5981,10 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="14" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C24" s="14"/>
       <c r="D24" s="14" t="s">
@@ -6000,10 +6000,10 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="14" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C25" s="14"/>
       <c r="D25" s="14" t="s">
@@ -6019,10 +6019,10 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="14" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C26" s="14"/>
       <c r="D26" s="14" t="s">
@@ -6038,10 +6038,10 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="14" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C27" s="14"/>
       <c r="D27" s="14" t="s">
@@ -6057,10 +6057,10 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" s="14" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C28" s="14"/>
       <c r="D28" s="14" t="s">
@@ -6076,10 +6076,10 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" s="14" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C29" s="14"/>
       <c r="D29" s="14" t="s">
@@ -6095,10 +6095,10 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="14" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C30" s="14"/>
       <c r="D30" s="14" t="s">
@@ -6133,10 +6133,10 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" s="14" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C32" s="14"/>
       <c r="D32" s="14" t="s">
@@ -6152,10 +6152,10 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" s="14" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C33" s="14"/>
       <c r="D33" s="14" t="s">
@@ -6190,13 +6190,13 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" s="14" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D35" s="14" t="s">
         <v>11</v>
@@ -6213,10 +6213,10 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" s="14" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C36" s="14"/>
       <c r="D36" s="14" t="s">
@@ -6232,10 +6232,10 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" s="14" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C37" s="14"/>
       <c r="D37" s="14" t="s">
@@ -6251,10 +6251,10 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" s="14" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C38" s="14"/>
       <c r="D38" s="14" t="s">
@@ -6270,10 +6270,10 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" s="14" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C39" s="14"/>
       <c r="D39" s="14" t="s">
@@ -6289,10 +6289,10 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" s="14" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C40" s="14"/>
       <c r="D40" s="14" t="s">
@@ -6308,10 +6308,10 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" s="14" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C41" s="14"/>
       <c r="D41" s="14" t="s">
@@ -6327,10 +6327,10 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" s="14" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C42" s="14"/>
       <c r="D42" s="14" t="s">
@@ -6367,7 +6367,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="17" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B1" s="17" t="s">
         <v>232</v>
@@ -6376,7 +6376,7 @@
         <v>151</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -6390,7 +6390,7 @@
         <v>105612</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -6404,7 +6404,7 @@
         <v>183279</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -6418,7 +6418,7 @@
         <v>41411</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -6432,7 +6432,7 @@
         <v>57146</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="E5" s="28"/>
     </row>
@@ -6447,7 +6447,7 @@
         <v>58758</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -6461,7 +6461,7 @@
         <v>16166</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="E7" s="30"/>
     </row>
@@ -6476,7 +6476,7 @@
         <v>26868</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="E8" s="30"/>
     </row>
@@ -6491,7 +6491,7 @@
         <v>30531</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="E9" s="30"/>
     </row>
@@ -6506,7 +6506,7 @@
         <v>17884</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="E10" s="30"/>
     </row>
@@ -6521,7 +6521,7 @@
         <v>33432</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="E11" s="30"/>
     </row>
@@ -6536,7 +6536,7 @@
         <v>83518</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="E12" s="30"/>
     </row>
@@ -6551,7 +6551,7 @@
         <v>8448</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="E13" s="30"/>
     </row>
@@ -6566,7 +6566,7 @@
         <v>56072</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="E14" s="30"/>
     </row>
@@ -6581,7 +6581,7 @@
         <v>67256</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="E15" s="30"/>
     </row>
@@ -6596,7 +6596,7 @@
         <v>16695</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -6610,7 +6610,7 @@
         <v>7482</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -6624,7 +6624,7 @@
         <v>21809</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -6638,7 +6638,7 @@
         <v>28695</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="E19" s="28"/>
     </row>
@@ -6653,7 +6653,7 @@
         <v>21939</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="E20" s="31"/>
     </row>
@@ -6668,7 +6668,7 @@
         <v>26700</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>